<commit_message>
feat: import category support
</commit_message>
<xml_diff>
--- a/admin/templates/notes-import-template.xlsx
+++ b/admin/templates/notes-import-template.xlsx
@@ -48,7 +48,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -56,27 +56,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -445,17 +431,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,30 +458,35 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>栏目</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>菜单简介</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>文首说明</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>章节标题</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>角标</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>块类型</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
@@ -513,32 +505,37 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Excel模板示例文章</t>
+          <t>学习</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>这是用Excel模板导入的示例</t>
+          <t>Excel模板示例</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>用Excel导入的示例</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>第一节：入门</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>p</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>这里写普通段落说明。</t>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>普通段落</t>
         </is>
       </c>
     </row>
@@ -555,32 +552,37 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Excel模板示例文章</t>
+          <t>学习</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>这是用Excel模板导入的示例</t>
+          <t>Excel模板示例</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>用Excel导入的示例</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>第一节：入门</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>h3</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>小标题示例</t>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>小标题</t>
         </is>
       </c>
     </row>
@@ -597,32 +599,37 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Excel模板示例文章</t>
+          <t>学习</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>这是用Excel模板导入的示例</t>
+          <t>Excel模板示例</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>用Excel导入的示例</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>第一节：入门</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>code</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>SELECT TOP 10 * FROM dbo.tb_bas_mold;</t>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>SELECT 1;</t>
         </is>
       </c>
     </row>
@@ -639,32 +646,37 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Excel模板示例文章</t>
+          <t>学习</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>这是用Excel模板导入的示例</t>
+          <t>Excel模板示例</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>用Excel导入的示例</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>第一节：入门</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>tip</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>提示类内容写在这里</t>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>提示内容</t>
         </is>
       </c>
     </row>
@@ -681,158 +693,84 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Excel模板示例文章</t>
+          <t>学习</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>这是用Excel模板导入的示例</t>
+          <t>Excel模板示例</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>用Excel导入的示例</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>第一节：入门</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>ul</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>条目A;;条目B;;条目C</t>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>条目A;;条目B</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>demo-office</t>
+          <t>demo-work</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Office导入示例</t>
+          <t>工作示例</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Excel模板示例文章</t>
+          <t>工作</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>这是用Excel模板导入的示例</t>
+          <t>工作栏目示例</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>第二节：进阶</t>
+          <t>工作相关说明</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>第一节</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>信息框示例</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>demo-office</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Office导入示例</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Excel模板示例文章</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>这是用Excel模板导入的示例</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>第二节：进阶</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>warning</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>注意风险事项</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>demo-office</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Office导入示例</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Excel模板示例文章</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>这是用Excel模板导入的示例</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>第二节：进阶</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
           <t>p</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>同一章节标题会自动合并为一节折叠卡片。</t>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>工作内容写在这里</t>
         </is>
       </c>
     </row>
@@ -847,7 +785,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -863,49 +801,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. 一块内容占一行。同一「文章ID」合并为一篇文章；同一「章节标题」合并为一节折叠卡片。</t>
+          <t>1. 栏目可填：工作 / 学习 / 娱乐（或栏目英文ID：work / study / fun）。留空则用导入区所选默认栏目。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2. 块类型可选：p（段落）/ h3（小标题）/ code（代码）/ tip / warning / info / ul（列表）</t>
+          <t>2. 同一文章ID合并为一篇；同一章节标题合并为一节折叠卡片。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>3. ul 的内容用英文双分号 ;; 分隔多个列表项，例如：项1;;项2;;项3</t>
+          <t>3. 块类型：p / h3 / code / tip / warning / info / ul；ul 用 ;; 分隔多项。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4. 文章ID 仅允许英文、数字、下划线、短横线。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>5. 角标可空，空则按章节顺序自动编号。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>6. 多篇文章可写在同一张表，用不同文章ID区分。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>7. 导入后可在管理后台再改为「私密」并设置密码。</t>
+          <t>4. 文章ID仅允许英文数字下划线短横线。</t>
         </is>
       </c>
     </row>

</xml_diff>